<commit_message>
Fix normalization pipeline v5 fixture contract
</commit_message>
<xml_diff>
--- a/tests/fixtures/normalization_bundle_minimal.xlsx
+++ b/tests/fixtures/normalization_bundle_minimal.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS Raw Records" sheetId="1" r:id="Rdcaf7922ab4a49cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalized Results" sheetId="2" r:id="R05e9de1d655047a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Rules" sheetId="3" r:id="Rb1154564349a4d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Manufacturer Catalog" sheetId="4" r:id="Rcd5922e138364d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effective Mfr Entities" sheetId="5" r:id="Rb13521296c3647a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Overrides" sheetId="6" r:id="R88d981a9d4a145c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Overrides" sheetId="7" r:id="Rdeb4eee8ee524388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Version" sheetId="8" r:id="R1bf19a9c06654828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS Raw Records" sheetId="1" r:id="Rbab113ca319a4adb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalized Results" sheetId="2" r:id="Rd94b8ca6539f4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Rules" sheetId="3" r:id="R231f60b173b549cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Manufacturer Catalog" sheetId="4" r:id="R85a1d6d0cfd84e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effective Mfr Entities" sheetId="5" r:id="R141d7b9d9da44ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Overrides" sheetId="6" r:id="Rab152c83d2694ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Overrides" sheetId="7" r:id="Rd3c59e9bf3c949f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Version" sheetId="8" r:id="R5c8c5b68857b4719"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb586a6764b054203"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfccc8816ba0c42fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -444,11 +444,41 @@
       <x:c r="A1" s="2" t="str">
         <x:v>Normalized Results</x:v>
       </x:c>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
+      <x:c r="G1"/>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
+      <x:c r="J1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
         <x:v>Deterministic integration-test fixture</x:v>
       </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6" t="str">
@@ -496,13 +526,13 @@
         <x:v>ts-review-fixture-v1</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>normalization-pipeline-v4</x:v>
+        <x:v>normalization-pipeline-v5</x:v>
       </x:c>
       <x:c r="F5" t="str">
         <x:v>review_required</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>{"normalized":{"market":["SE"],"alias_types_present":["plate","vin","model_name"],"manufacturer":"Volvo","manufacturer_role":"vehicle_manufacturer","builder_converter_names":[],"model_family_candidate":true,"power_kw":145,"power_source_unit":"kw","displacement_cc":1969,"displacement_source_unit":"ccm","transmission_type":"automatic","bodywork_registry_label_sv":"Stationsvagn (kombivagn)","bodywork_form":"estate"},"candidates":{"model_family":"V60"},"candidate_rule_ids":[],"confidence":0.55,"pipeline_version":"normalization-pipeline-v4","decision_trace":[{"sequence":1,"transformer_id":"ts.initialize","target":"normalized","field":"alias_types_present","rule_ids":["SYS-TS-INIT"],"before":null,"after":["plate","vin","model_name"],"confidence_effect":0.0},{"sequence":2,"transformer_id":"ts.initialize","target":"normalized","field":"market","rule_ids":["SYS-TS-INIT"],"before":null,"after":["SE"],"confidence_effect":0.0},{"sequence":3,"transformer_id":"ts.manufacturer","target":"normalized","field":"builder_converter_names","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":[],"confidence_effect":0.2},{"sequence":4,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"Volvo","confidence_effect":0.2},{"sequence":5,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_role","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"vehicle_manufacturer","confidence_effect":0.2},{"sequence":6,"transformer_id":"ts.model-family","target":"normalized","field":"model_family_candidate","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":true,"confidence_effect":0.0},{"sequence":7,"transformer_id":"ts.model-family","target":"candidate","field":"model_family","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":"V60","confidence_effect":0.05},{"sequence":8,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_cc","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":1969,"confidence_effect":0.1},{"sequence":9,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"ccm","confidence_effect":0.1},{"sequence":10,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_kw","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":145,"confidence_effect":0.1},{"sequence":11,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"kw","confidence_effect":0.1},{"sequence":12,"transformer_id":"ts.transmission","target":"normalized","field":"transmission_type","rule_ids":["TRN-008"],"before":{"gearbox":"Z","model":"V60"},"after":"automatic","confidence_effect":0.1},{"sequence":13,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_form","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"estate","confidence_effect":0.1},{"sequence":14,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_label_sv","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"Stationsvagn (kombivagn)","confidence_effect":0.1},{"sequence":15,"transformer_id":"ts.fuel","target":"review","field":"review_reason","rule_ids":["FUEL-LOOKUP-V1"],"before":{"fuel1":"BENSIN","model":"V60"},"after":"fuel1_code_unknown","confidence_effect":-0.2}],"rule_matches":[{"rule_set_version":"ts-review-fixture-v1","rule_id":"TRN-008","decision":"accepted","source_field":"gearbox","source_term":"Z","target_field":"transmission_type","canonical_value":"automatic"},{"rule_set_version":"ts-review-fixture-v1","rule_id":"BDY-110","decision":"accepted","source_field":"body_code","source_term":"AC","target_field":"bodywork_form","canonical_value":"estate"}]}</x:v>
+        <x:v>{"normalized":{"market":["SE"],"alias_types_present":["plate","vin","model_name"],"legal_manufacturer":"VOLVO CAR CORPORATION","manufacturer":"Volvo","manufacturer_role":"vehicle_manufacturer","builder_converter_names":[],"manufacturer_evidence":["manufacturer"],"model_family_candidate":true,"power_kw":145,"power_source_unit":"kw","displacement_cc":1969,"displacement_source_unit":"ccm","transmission_type":"automatic","bodywork_registry_code":"AC","bodywork_registry_label_sv":"Stationsvagn (kombivagn)","bodywork_form":"estate","bodywork_source":"registry"},"candidates":{"model_family":"V60"},"confidence":0.55,"pipeline_version":"normalization-pipeline-v5","decision_trace":[{"sequence":1,"transformer_id":"ts.initialize","target":"normalized","field":"alias_types_present","rule_ids":["SYS-TS-INIT"],"before":null,"after":["plate","vin","model_name"],"confidence_effect":0},{"sequence":2,"transformer_id":"ts.initialize","target":"normalized","field":"market","rule_ids":["SYS-TS-INIT"],"before":null,"after":["SE"],"confidence_effect":0},{"sequence":3,"transformer_id":"ts.manufacturer","target":"normalized","field":"builder_converter_names","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":[],"confidence_effect":0.2},{"sequence":4,"transformer_id":"ts.manufacturer","target":"normalized","field":"legal_manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"VOLVO CAR CORPORATION","confidence_effect":0.2},{"sequence":5,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"Volvo","confidence_effect":0.2},{"sequence":6,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_evidence","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":["manufacturer"],"confidence_effect":0.2},{"sequence":7,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_role","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"vehicle_manufacturer","confidence_effect":0.2},{"sequence":8,"transformer_id":"ts.model-family","target":"normalized","field":"model_family_candidate","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":true,"confidence_effect":0},{"sequence":9,"transformer_id":"ts.model-family","target":"candidate","field":"model_family","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":"V60","confidence_effect":0.05},{"sequence":10,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_cc","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":1969,"confidence_effect":0.1},{"sequence":11,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"ccm","confidence_effect":0.1},{"sequence":12,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_kw","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":145,"confidence_effect":0.1},{"sequence":13,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"kw","confidence_effect":0.1},{"sequence":14,"transformer_id":"ts.transmission","target":"normalized","field":"transmission_type","rule_ids":["TRN-008"],"before":{"gearbox":"Z","model":"V60"},"after":"automatic","confidence_effect":0.1},{"sequence":15,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_form","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"estate","confidence_effect":0.1},{"sequence":16,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_code","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"AC","confidence_effect":0.1},{"sequence":17,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_label_sv","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"Stationsvagn (kombivagn)","confidence_effect":0.1},{"sequence":18,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_source","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"registry","confidence_effect":0.1},{"sequence":19,"transformer_id":"ts.fuel","target":"review","field":"review_reason","rule_ids":["FUEL-LOOKUP-V1"],"before":{"fuel1":"BENSIN","model":"V60"},"after":"fuel1_code_unknown","confidence_effect":-0.2}],"rule_matches":[{"rule_set_version":"ts-review-fixture-v1","rule_id":"TRN-008","decision":"accepted","source_field":"gearbox","source_term":"Z","target_field":"transmission_type","canonical_value":"automatic"},{"rule_set_version":"ts-review-fixture-v1","rule_id":"BDY-110","decision":"accepted","source_field":"body_code","source_term":"AC","target_field":"bodywork_form","canonical_value":"estate"}]}</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>["MFR-102","UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1","TRN-008","BDY-110"]</x:v>
@@ -521,7 +551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0570324d2ec46a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R498a687ef5b74ecd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -538,11 +568,17 @@
       <x:c r="A1" s="2" t="str">
         <x:v>Translation Rules</x:v>
       </x:c>
+      <x:c r="B1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
         <x:v>Deterministic integration-test fixture</x:v>
       </x:c>
+      <x:c r="B2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6" t="str">
@@ -581,7 +617,7 @@
         <x:v>BDY-004</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>{"rule_id":"BDY-004","area":"bodywork_marketing","source_fields":["model","variant","version","type"],"source_terms":["Estate","Wagon","Kombi","Break","Sport Tourer","Shooting Brake","SW"],"canonical_field":"bodywork_form","canonical_value":"estate","decision":"accepted","display_value":null,"vehicle_scopes":[],"manufacturers":["*"],"requires_electrification":false}</x:v>
+        <x:v>{"rule_id":"BDY-004","area":"bodywork_marketing","source_fields":["model","variant","version","type"],"source_terms":["Estate","Wagon","Kombi","Combi","Break","Sport Tourer","Shooting Brake","SW"],"canonical_field":"bodywork_form","canonical_value":"estate","decision":"accepted","display_value":null,"vehicle_scopes":[],"manufacturers":["*"],"requires_electrification":false}</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1351,7 +1387,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d6da4a02a934b02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd0f94ff08b54c73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2861,7 +2897,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10d808959b8d4b57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0bc0f7b5b64b8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4371,7 +4407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa0aeda3be584057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9dadc46c9c1432a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4515,7 +4551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R476cd22b9cc14cdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eb61a8b6e5f4bee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Include candidate rule IDs in v5 fixture
</commit_message>
<xml_diff>
--- a/tests/fixtures/normalization_bundle_minimal.xlsx
+++ b/tests/fixtures/normalization_bundle_minimal.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS Raw Records" sheetId="1" r:id="Rbab113ca319a4adb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalized Results" sheetId="2" r:id="Rd94b8ca6539f4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Rules" sheetId="3" r:id="R231f60b173b549cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Manufacturer Catalog" sheetId="4" r:id="R85a1d6d0cfd84e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effective Mfr Entities" sheetId="5" r:id="R141d7b9d9da44ebf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Overrides" sheetId="6" r:id="Rab152c83d2694ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Overrides" sheetId="7" r:id="Rd3c59e9bf3c949f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Version" sheetId="8" r:id="R5c8c5b68857b4719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS Raw Records" sheetId="1" r:id="R1209de7e73d94d75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalized Results" sheetId="2" r:id="Rce2fffade3324033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Rules" sheetId="3" r:id="Ra4734d246a2b4fa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Manufacturer Catalog" sheetId="4" r:id="Re8111767ef0142f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effective Mfr Entities" sheetId="5" r:id="R4298921c983a40bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Overrides" sheetId="6" r:id="R46eea64f48364bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Overrides" sheetId="7" r:id="R4c31de6f0ea340a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Version" sheetId="8" r:id="Rb42aceb35f0d4f32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfccc8816ba0c42fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea42fa170bd4244"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -532,7 +532,7 @@
         <x:v>review_required</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>{"normalized":{"market":["SE"],"alias_types_present":["plate","vin","model_name"],"legal_manufacturer":"VOLVO CAR CORPORATION","manufacturer":"Volvo","manufacturer_role":"vehicle_manufacturer","builder_converter_names":[],"manufacturer_evidence":["manufacturer"],"model_family_candidate":true,"power_kw":145,"power_source_unit":"kw","displacement_cc":1969,"displacement_source_unit":"ccm","transmission_type":"automatic","bodywork_registry_code":"AC","bodywork_registry_label_sv":"Stationsvagn (kombivagn)","bodywork_form":"estate","bodywork_source":"registry"},"candidates":{"model_family":"V60"},"confidence":0.55,"pipeline_version":"normalization-pipeline-v5","decision_trace":[{"sequence":1,"transformer_id":"ts.initialize","target":"normalized","field":"alias_types_present","rule_ids":["SYS-TS-INIT"],"before":null,"after":["plate","vin","model_name"],"confidence_effect":0},{"sequence":2,"transformer_id":"ts.initialize","target":"normalized","field":"market","rule_ids":["SYS-TS-INIT"],"before":null,"after":["SE"],"confidence_effect":0},{"sequence":3,"transformer_id":"ts.manufacturer","target":"normalized","field":"builder_converter_names","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":[],"confidence_effect":0.2},{"sequence":4,"transformer_id":"ts.manufacturer","target":"normalized","field":"legal_manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"VOLVO CAR CORPORATION","confidence_effect":0.2},{"sequence":5,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"Volvo","confidence_effect":0.2},{"sequence":6,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_evidence","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":["manufacturer"],"confidence_effect":0.2},{"sequence":7,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_role","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"vehicle_manufacturer","confidence_effect":0.2},{"sequence":8,"transformer_id":"ts.model-family","target":"normalized","field":"model_family_candidate","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":true,"confidence_effect":0},{"sequence":9,"transformer_id":"ts.model-family","target":"candidate","field":"model_family","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":"V60","confidence_effect":0.05},{"sequence":10,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_cc","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":1969,"confidence_effect":0.1},{"sequence":11,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"ccm","confidence_effect":0.1},{"sequence":12,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_kw","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":145,"confidence_effect":0.1},{"sequence":13,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"kw","confidence_effect":0.1},{"sequence":14,"transformer_id":"ts.transmission","target":"normalized","field":"transmission_type","rule_ids":["TRN-008"],"before":{"gearbox":"Z","model":"V60"},"after":"automatic","confidence_effect":0.1},{"sequence":15,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_form","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"estate","confidence_effect":0.1},{"sequence":16,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_code","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"AC","confidence_effect":0.1},{"sequence":17,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_label_sv","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"Stationsvagn (kombivagn)","confidence_effect":0.1},{"sequence":18,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_source","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"registry","confidence_effect":0.1},{"sequence":19,"transformer_id":"ts.fuel","target":"review","field":"review_reason","rule_ids":["FUEL-LOOKUP-V1"],"before":{"fuel1":"BENSIN","model":"V60"},"after":"fuel1_code_unknown","confidence_effect":-0.2}],"rule_matches":[{"rule_set_version":"ts-review-fixture-v1","rule_id":"TRN-008","decision":"accepted","source_field":"gearbox","source_term":"Z","target_field":"transmission_type","canonical_value":"automatic"},{"rule_set_version":"ts-review-fixture-v1","rule_id":"BDY-110","decision":"accepted","source_field":"body_code","source_term":"AC","target_field":"bodywork_form","canonical_value":"estate"}]}</x:v>
+        <x:v>{"normalized":{"market":["SE"],"alias_types_present":["plate","vin","model_name"],"legal_manufacturer":"VOLVO CAR CORPORATION","manufacturer":"Volvo","manufacturer_role":"vehicle_manufacturer","builder_converter_names":[],"manufacturer_evidence":["manufacturer"],"model_family_candidate":true,"power_kw":145,"power_source_unit":"kw","displacement_cc":1969,"displacement_source_unit":"ccm","transmission_type":"automatic","bodywork_registry_code":"AC","bodywork_registry_label_sv":"Stationsvagn (kombivagn)","bodywork_form":"estate","bodywork_source":"registry"},"candidates":{"model_family":"V60"},"confidence":0.55,"pipeline_version":"normalization-pipeline-v5","decision_trace":[{"sequence":1,"transformer_id":"ts.initialize","target":"normalized","field":"alias_types_present","rule_ids":["SYS-TS-INIT"],"before":null,"after":["plate","vin","model_name"],"confidence_effect":0},{"sequence":2,"transformer_id":"ts.initialize","target":"normalized","field":"market","rule_ids":["SYS-TS-INIT"],"before":null,"after":["SE"],"confidence_effect":0},{"sequence":3,"transformer_id":"ts.manufacturer","target":"normalized","field":"builder_converter_names","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":[],"confidence_effect":0.2},{"sequence":4,"transformer_id":"ts.manufacturer","target":"normalized","field":"legal_manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"VOLVO CAR CORPORATION","confidence_effect":0.2},{"sequence":5,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"Volvo","confidence_effect":0.2},{"sequence":6,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_evidence","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":["manufacturer"],"confidence_effect":0.2},{"sequence":7,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_role","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"vehicle_manufacturer","confidence_effect":0.2},{"sequence":8,"transformer_id":"ts.model-family","target":"normalized","field":"model_family_candidate","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":true,"confidence_effect":0},{"sequence":9,"transformer_id":"ts.model-family","target":"candidate","field":"model_family","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":"V60","confidence_effect":0.05},{"sequence":10,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_cc","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":1969,"confidence_effect":0.1},{"sequence":11,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"ccm","confidence_effect":0.1},{"sequence":12,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_kw","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":145,"confidence_effect":0.1},{"sequence":13,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"kw","confidence_effect":0.1},{"sequence":14,"transformer_id":"ts.transmission","target":"normalized","field":"transmission_type","rule_ids":["TRN-008"],"before":{"gearbox":"Z","model":"V60"},"after":"automatic","confidence_effect":0.1},{"sequence":15,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_form","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"estate","confidence_effect":0.1},{"sequence":16,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_code","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"AC","confidence_effect":0.1},{"sequence":17,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_label_sv","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"Stationsvagn (kombivagn)","confidence_effect":0.1},{"sequence":18,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_source","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"registry","confidence_effect":0.1},{"sequence":19,"transformer_id":"ts.fuel","target":"review","field":"review_reason","rule_ids":["FUEL-LOOKUP-V1"],"before":{"fuel1":"BENSIN","model":"V60"},"after":"fuel1_code_unknown","confidence_effect":-0.2}],"rule_matches":[{"rule_set_version":"ts-review-fixture-v1","rule_id":"TRN-008","decision":"accepted","source_field":"gearbox","source_term":"Z","target_field":"transmission_type","canonical_value":"automatic"},{"rule_set_version":"ts-review-fixture-v1","rule_id":"BDY-110","decision":"accepted","source_field":"body_code","source_term":"AC","target_field":"bodywork_form","canonical_value":"estate"}],"candidate_rule_ids":[]}</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>["MFR-102","UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1","TRN-008","BDY-110"]</x:v>
@@ -551,7 +551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R498a687ef5b74ecd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R194e1233e1a14a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1387,7 +1387,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd0f94ff08b54c73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a83ad340014a5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2897,7 +2897,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0bc0f7b5b64b8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27a91713bee14a68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4407,7 +4407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9dadc46c9c1432a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1c3511a1544c31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4551,7 +4551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eb61a8b6e5f4bee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc64a47dd6349483d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix normalization bundle confidence trace
</commit_message>
<xml_diff>
--- a/tests/fixtures/normalization_bundle_minimal.xlsx
+++ b/tests/fixtures/normalization_bundle_minimal.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS Raw Records" sheetId="1" r:id="R1209de7e73d94d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalized Results" sheetId="2" r:id="Rce2fffade3324033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Rules" sheetId="3" r:id="Ra4734d246a2b4fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Manufacturer Catalog" sheetId="4" r:id="Re8111767ef0142f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effective Mfr Entities" sheetId="5" r:id="R4298921c983a40bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Overrides" sheetId="6" r:id="R46eea64f48364bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Overrides" sheetId="7" r:id="R4c31de6f0ea340a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Version" sheetId="8" r:id="Rb42aceb35f0d4f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS Raw Records" sheetId="1" r:id="Re3c054d7ae534ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalized Results" sheetId="2" r:id="Rdc6a03ec0c5e4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Rules" sheetId="3" r:id="Ra7bc33b2de8d4d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Manufacturer Catalog" sheetId="4" r:id="R474012d07fbb46f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effective Mfr Entities" sheetId="5" r:id="R9a26532da1f544a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Overrides" sheetId="6" r:id="R093fb44b06764f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Overrides" sheetId="7" r:id="R63ceb8b51b5e4fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Version" sheetId="8" r:id="R0e4b03c4a50146b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea42fa170bd4244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2cedce52c5f466e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -532,7 +532,7 @@
         <x:v>review_required</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>{"normalized":{"market":["SE"],"alias_types_present":["plate","vin","model_name"],"legal_manufacturer":"VOLVO CAR CORPORATION","manufacturer":"Volvo","manufacturer_role":"vehicle_manufacturer","builder_converter_names":[],"manufacturer_evidence":["manufacturer"],"model_family_candidate":true,"power_kw":145,"power_source_unit":"kw","displacement_cc":1969,"displacement_source_unit":"ccm","transmission_type":"automatic","bodywork_registry_code":"AC","bodywork_registry_label_sv":"Stationsvagn (kombivagn)","bodywork_form":"estate","bodywork_source":"registry"},"candidates":{"model_family":"V60"},"confidence":0.55,"pipeline_version":"normalization-pipeline-v5","decision_trace":[{"sequence":1,"transformer_id":"ts.initialize","target":"normalized","field":"alias_types_present","rule_ids":["SYS-TS-INIT"],"before":null,"after":["plate","vin","model_name"],"confidence_effect":0},{"sequence":2,"transformer_id":"ts.initialize","target":"normalized","field":"market","rule_ids":["SYS-TS-INIT"],"before":null,"after":["SE"],"confidence_effect":0},{"sequence":3,"transformer_id":"ts.manufacturer","target":"normalized","field":"builder_converter_names","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":[],"confidence_effect":0.2},{"sequence":4,"transformer_id":"ts.manufacturer","target":"normalized","field":"legal_manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"VOLVO CAR CORPORATION","confidence_effect":0.2},{"sequence":5,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"Volvo","confidence_effect":0.2},{"sequence":6,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_evidence","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":["manufacturer"],"confidence_effect":0.2},{"sequence":7,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_role","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"vehicle_manufacturer","confidence_effect":0.2},{"sequence":8,"transformer_id":"ts.model-family","target":"normalized","field":"model_family_candidate","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":true,"confidence_effect":0},{"sequence":9,"transformer_id":"ts.model-family","target":"candidate","field":"model_family","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":"V60","confidence_effect":0.05},{"sequence":10,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_cc","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":1969,"confidence_effect":0.1},{"sequence":11,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"ccm","confidence_effect":0.1},{"sequence":12,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_kw","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":145,"confidence_effect":0.1},{"sequence":13,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"kw","confidence_effect":0.1},{"sequence":14,"transformer_id":"ts.transmission","target":"normalized","field":"transmission_type","rule_ids":["TRN-008"],"before":{"gearbox":"Z","model":"V60"},"after":"automatic","confidence_effect":0.1},{"sequence":15,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_form","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"estate","confidence_effect":0.1},{"sequence":16,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_code","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"AC","confidence_effect":0.1},{"sequence":17,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_label_sv","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"Stationsvagn (kombivagn)","confidence_effect":0.1},{"sequence":18,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_source","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"registry","confidence_effect":0.1},{"sequence":19,"transformer_id":"ts.fuel","target":"review","field":"review_reason","rule_ids":["FUEL-LOOKUP-V1"],"before":{"fuel1":"BENSIN","model":"V60"},"after":"fuel1_code_unknown","confidence_effect":-0.2}],"rule_matches":[{"rule_set_version":"ts-review-fixture-v1","rule_id":"TRN-008","decision":"accepted","source_field":"gearbox","source_term":"Z","target_field":"transmission_type","canonical_value":"automatic"},{"rule_set_version":"ts-review-fixture-v1","rule_id":"BDY-110","decision":"accepted","source_field":"body_code","source_term":"AC","target_field":"bodywork_form","canonical_value":"estate"}],"candidate_rule_ids":[]}</x:v>
+        <x:v>{"normalized":{"market":["SE"],"alias_types_present":["plate","vin","model_name"],"legal_manufacturer":"VOLVO CAR CORPORATION","manufacturer":"Volvo","manufacturer_role":"vehicle_manufacturer","builder_converter_names":[],"manufacturer_evidence":["manufacturer"],"model_family_candidate":true,"power_kw":145,"power_source_unit":"kw","displacement_cc":1969,"displacement_source_unit":"ccm","transmission_type":"automatic","bodywork_registry_code":"AC","bodywork_registry_label_sv":"Stationsvagn (kombivagn)","bodywork_form":"estate","bodywork_source":"registry"},"candidates":{"model_family":"V60"},"confidence":0.55,"pipeline_version":"normalization-pipeline-v5","decision_trace":[{"sequence":1,"transformer_id":"ts.initialize","target":"normalized","field":"alias_types_present","rule_ids":["SYS-TS-INIT"],"before":null,"after":["plate","vin","model_name"],"confidence_effect":0},{"sequence":2,"transformer_id":"ts.initialize","target":"normalized","field":"market","rule_ids":["SYS-TS-INIT"],"before":null,"after":["SE"],"confidence_effect":0},{"sequence":3,"transformer_id":"ts.manufacturer","target":"normalized","field":"builder_converter_names","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":[],"confidence_effect":0.2},{"sequence":4,"transformer_id":"ts.manufacturer","target":"normalized","field":"legal_manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"VOLVO CAR CORPORATION","confidence_effect":0.2},{"sequence":5,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"Volvo","confidence_effect":0.2},{"sequence":6,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_evidence","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":["manufacturer"],"confidence_effect":0.2},{"sequence":7,"transformer_id":"ts.manufacturer","target":"normalized","field":"manufacturer_role","rule_ids":["MFR-102"],"before":"VOLVO CAR CORPORATION","after":"vehicle_manufacturer","confidence_effect":0.2},{"sequence":8,"transformer_id":"ts.model-family","target":"normalized","field":"model_family_candidate","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":true,"confidence_effect":0.1},{"sequence":9,"transformer_id":"ts.model-family","target":"candidate","field":"model_family","rule_ids":["MODEL-CANDIDATE-V1"],"before":"V60","after":"V60","confidence_effect":0.05},{"sequence":10,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_cc","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":1969,"confidence_effect":0.1},{"sequence":11,"transformer_id":"ts.engine-measurements","target":"normalized","field":"displacement_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"ccm","confidence_effect":0.1},{"sequence":12,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_kw","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":145,"confidence_effect":0.1},{"sequence":13,"transformer_id":"ts.engine-measurements","target":"normalized","field":"power_source_unit","rule_ids":["UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1"],"before":{"kw":145,"ccm":1969},"after":"kw","confidence_effect":0.1},{"sequence":14,"transformer_id":"ts.transmission","target":"normalized","field":"transmission_type","rule_ids":["TRN-008"],"before":{"gearbox":"Z","model":"V60"},"after":"automatic","confidence_effect":0.1},{"sequence":15,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_form","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"estate","confidence_effect":0.1},{"sequence":16,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_code","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"AC","confidence_effect":0.1},{"sequence":17,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_registry_label_sv","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"Stationsvagn (kombivagn)","confidence_effect":0.1},{"sequence":18,"transformer_id":"ts.bodywork","target":"normalized","field":"bodywork_source","rule_ids":["BDY-110"],"before":{"body_code":"AC","eu_category":"M1","model":"V60"},"after":"registry","confidence_effect":0.1},{"sequence":19,"transformer_id":"ts.fuel","target":"review","field":"review_reason","rule_ids":["FUEL-LOOKUP-V1"],"before":{"fuel1":"BENSIN","model":"V60"},"after":"fuel1_code_unknown","confidence_effect":-0.2}],"rule_matches":[{"rule_set_version":"ts-review-fixture-v1","rule_id":"TRN-008","decision":"accepted","source_field":"gearbox","source_term":"Z","target_field":"transmission_type","canonical_value":"automatic"},{"rule_set_version":"ts-review-fixture-v1","rule_id":"BDY-110","decision":"accepted","source_field":"body_code","source_term":"AC","target_field":"bodywork_form","canonical_value":"estate"}],"candidate_rule_ids":[]}</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>["MFR-102","UNIT-POWER-KW-V1","UNIT-DISPLACEMENT-CCM-V1","TRN-008","BDY-110"]</x:v>
@@ -551,7 +551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R194e1233e1a14a78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde2d8a611b46484a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1387,7 +1387,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a83ad340014a5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0163db688a844a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2897,7 +2897,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27a91713bee14a68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf364c03da5f4662"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4407,7 +4407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1c3511a1544c31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1da86fe59a1f47f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4551,7 +4551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc64a47dd6349483d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8372ed7a7b1f4c66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>